<commit_message>
Update README.md for clarity and enhance documentation structure
</commit_message>
<xml_diff>
--- a/output/documentation.xlsx
+++ b/output/documentation.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="16">
   <si>
     <t>File Name</t>
   </si>
@@ -32,19 +32,16 @@
     <t>Module</t>
   </si>
   <si>
-    <t>run.go</t>
-  </si>
-  <si>
-    <t>internal/cli/run.go</t>
+    <t>README.md</t>
   </si>
   <si>
     <t>Modified</t>
   </si>
   <si>
-    <t>go</t>
-  </si>
-  <si>
-    <t>internal</t>
+    <t>md</t>
+  </si>
+  <si>
+    <t>root</t>
   </si>
   <si>
     <t>Metric</t>
@@ -394,16 +391,16 @@
         <v>5</v>
       </c>
       <c r="B2" t="s">
+        <v>5</v>
+      </c>
+      <c r="C2" t="s">
         <v>6</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>8</v>
-      </c>
-      <c r="E2" t="s">
-        <v>9</v>
       </c>
     </row>
   </sheetData>
@@ -416,42 +413,42 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B1" t="s">
         <v>10</v>
-      </c>
-      <c r="B1" t="s">
-        <v>11</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
+        <v>11</v>
+      </c>
+      <c r="B2" t="s">
         <v>12</v>
-      </c>
-      <c r="B2" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B5" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>

</xml_diff>